<commit_message>
Refine core audit engine and prepare production-ready scheduler architecture
</commit_message>
<xml_diff>
--- a/tracking_plan.xlsx
+++ b/tracking_plan.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,6 +78,9 @@
       <name val="Arial"/>
       <color rgb="001E293B"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -144,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -182,6 +185,7 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1775,7 +1779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2890,90 +2894,158 @@
       <c r="H34" s="10" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Product Viewed</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>variant_id</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>var_998877</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>Shopify variant ID. Matches the variant selected by user.</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="n"/>
+    </row>
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Product Viewed</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>SKU-LIB-BLK-M</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>Merchant SKU string. Sent for cross-reference with inventory.</t>
+        </is>
+      </c>
+      <c r="H36" s="10" t="n"/>
+    </row>
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>▶ Size Chart Viewed</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>User opens the size guide modal on PDP.</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr"/>
-      <c r="D35" s="8" t="inlineStr"/>
-      <c r="E35" s="8" t="inlineStr"/>
-      <c r="F35" s="8" t="inlineStr"/>
-      <c r="G35" s="8" t="inlineStr"/>
-      <c r="H35" s="8" t="inlineStr"/>
-    </row>
-    <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr"/>
+      <c r="D37" s="8" t="inlineStr"/>
+      <c r="E37" s="8" t="inlineStr"/>
+      <c r="F37" s="8" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr"/>
+      <c r="H37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>Size Chart Viewed</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>SKU-BLK-M</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr"/>
-      <c r="G36" s="9" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr"/>
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>Product SKU.</t>
         </is>
       </c>
-      <c r="H36" s="9" t="inlineStr"/>
-    </row>
-    <row r="37" ht="34" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="H38" s="9" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Size Chart Viewed</t>
         </is>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>Women's Kurtas</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr"/>
-      <c r="G37" s="10" t="inlineStr">
+      <c r="F39" s="10" t="inlineStr"/>
+      <c r="G39" s="10" t="inlineStr">
         <is>
           <t>Category determines which size chart is shown.</t>
         </is>
       </c>
-      <c r="H37" s="10" t="inlineStr"/>
+      <c r="H39" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2990,7 +3062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3453,90 +3525,88 @@
       <c r="H14" s="10" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Product Added</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>variant_id</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>var_998877</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Shopify variant ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Product Added</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>SKU-LIB-BLK-M</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Merchant SKU string.</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="n"/>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>▶ Product Removed</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>User removes an item from cart.</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr"/>
-      <c r="D15" s="8" t="inlineStr"/>
-      <c r="E15" s="8" t="inlineStr"/>
-      <c r="F15" s="8" t="inlineStr"/>
-      <c r="G15" s="8" t="inlineStr"/>
-      <c r="H15" s="8" t="inlineStr"/>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Product Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>cart_id</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>cart_a1b2c3</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr"/>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Cart ID.</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Product Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>product_id</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>SKU-BLK-M</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr"/>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>SKU removed.</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr"/>
+      <c r="C17" s="8" t="inlineStr"/>
+      <c r="D17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr"/>
+      <c r="H17" s="8" t="inlineStr"/>
     </row>
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -3546,7 +3616,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>cart_id</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -3561,13 +3631,13 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Black Cotton Kurta</t>
+          <t>cart_a1b2c3</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr"/>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>Product title.</t>
+          <t>Cart ID.</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr"/>
@@ -3580,7 +3650,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>product_id</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -3590,18 +3660,18 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>799.00</t>
+          <t>SKU-BLK-M</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr"/>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>Unit price in INR.</t>
+          <t>SKU removed.</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr"/>
@@ -3614,7 +3684,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -3624,18 +3694,18 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Black Cotton Kurta</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr"/>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Quantity removed.</t>
+          <t>Product title.</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr"/>
@@ -3648,7 +3718,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>price</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -3658,53 +3728,65 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>INR</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
+          <t>799.00</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr"/>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>Always INR.</t>
+          <t>Unit price in INR.</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>▶ Cart Viewed</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>User opens the cart page or drawer.</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr"/>
-      <c r="D22" s="8" t="inlineStr"/>
-      <c r="E22" s="8" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr"/>
-      <c r="G22" s="8" t="inlineStr"/>
-      <c r="H22" s="8" t="inlineStr"/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Product Removed</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr"/>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Quantity removed.</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr"/>
     </row>
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Cart Viewed</t>
+          <t>Product Removed</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>cart_id</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -3719,50 +3801,38 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>cart_a1b2c3</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr"/>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Cart ID.</t>
+          <t>Always INR.</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr"/>
     </row>
     <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Cart Viewed</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>total_items</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr"/>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>Total item quantity in cart.</t>
-        </is>
-      </c>
-      <c r="H24" s="9" t="inlineStr"/>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>▶ Cart Viewed</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>User opens the cart page or drawer.</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr"/>
+      <c r="D24" s="8" t="inlineStr"/>
+      <c r="E24" s="8" t="inlineStr"/>
+      <c r="F24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr"/>
+      <c r="H24" s="8" t="inlineStr"/>
     </row>
     <row r="25" ht="34" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -3772,7 +3842,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>subtotal</t>
+          <t>cart_id</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -3782,18 +3852,18 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>1598.00</t>
+          <t>cart_a1b2c3</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr"/>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Cart subtotal before discounts and shipping in INR.</t>
+          <t>Cart ID.</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr"/>
@@ -3806,7 +3876,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>total_items</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -3816,53 +3886,65 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>INR</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr"/>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Always INR.</t>
+          <t>Total item quantity in cart.</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>▶ Checkout Started</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>User proceeds from cart to checkout. Segment Ecommerce standard.</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr"/>
-      <c r="D27" s="8" t="inlineStr"/>
-      <c r="E27" s="8" t="inlineStr"/>
-      <c r="F27" s="8" t="inlineStr"/>
-      <c r="G27" s="8" t="inlineStr"/>
-      <c r="H27" s="8" t="inlineStr"/>
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Cart Viewed</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>subtotal</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>1598.00</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr"/>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>Cart subtotal before discounts and shipping in INR.</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr"/>
     </row>
     <row r="28" ht="34" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Checkout Started</t>
+          <t>Cart Viewed</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>order_id</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -3877,50 +3959,38 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>ORD-20250401-9821</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="inlineStr"/>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>Pre-assigned draft order ID.</t>
+          <t>Always INR.</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr"/>
     </row>
     <row r="29" ht="34" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Checkout Started</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>cart_id</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>cart_a1b2c3</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="inlineStr"/>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>Cart ID.</t>
-        </is>
-      </c>
-      <c r="H29" s="9" t="inlineStr"/>
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>▶ Checkout Started</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>User proceeds from cart to checkout. Segment Ecommerce standard.</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr"/>
+      <c r="E29" s="8" t="inlineStr"/>
+      <c r="F29" s="8" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr"/>
+      <c r="H29" s="8" t="inlineStr"/>
     </row>
     <row r="30" ht="34" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
@@ -3930,7 +4000,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>revenue</t>
+          <t>order_id</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -3940,18 +4010,18 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>1598.00</t>
+          <t>ORD-20250401-9821</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr"/>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>Cart subtotal in INR.</t>
+          <t>Pre-assigned draft order ID.</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr"/>
@@ -3964,103 +4034,103 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
+          <t>cart_id</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>cart_a1b2c3</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr"/>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>Cart ID.</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr"/>
+    </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Checkout Started</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>1598.00</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr"/>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>Cart subtotal in INR.</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr"/>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>Checkout Started</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G33" s="9" t="inlineStr">
         <is>
           <t>Always INR.</t>
         </is>
       </c>
-      <c r="H31" s="9" t="inlineStr"/>
-    </row>
-    <row r="32" ht="34" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Checkout Started</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>coupon</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>FIRST10</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr"/>
-      <c r="G32" s="10" t="inlineStr">
-        <is>
-          <t>Coupon code applied, if any.</t>
-        </is>
-      </c>
-      <c r="H32" s="10" t="inlineStr"/>
-    </row>
-    <row r="33" ht="34" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Checkout Started</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>discount</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
-        <is>
-          <t>159.80</t>
-        </is>
-      </c>
-      <c r="F33" s="10" t="inlineStr"/>
-      <c r="G33" s="10" t="inlineStr">
-        <is>
-          <t>Discount amount in INR.</t>
-        </is>
-      </c>
-      <c r="H33" s="10" t="inlineStr"/>
+      <c r="H33" s="9" t="inlineStr"/>
     </row>
     <row r="34" ht="34" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
@@ -4070,7 +4140,7 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>num_items</t>
+          <t>coupon</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -4080,321 +4150,335 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>FIRST10</t>
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr"/>
       <c r="G34" s="10" t="inlineStr">
         <is>
+          <t>Coupon code applied, if any.</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Checkout Started</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>discount</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>159.80</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr"/>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>Discount amount in INR.</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="inlineStr"/>
+    </row>
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Checkout Started</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>num_items</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr"/>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
           <t>Total item count in checkout.</t>
         </is>
       </c>
-      <c r="H34" s="10" t="inlineStr"/>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="H36" s="10" t="inlineStr"/>
+    </row>
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Checkout Started</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>checkout_token</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>sh_9a8b7c6d</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Shopify checkout token.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="34" customHeight="1">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>▶ Checkout Step Completed</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>User completes a checkout step and advances to the next.</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr"/>
-      <c r="D35" s="8" t="inlineStr"/>
-      <c r="E35" s="8" t="inlineStr"/>
-      <c r="F35" s="8" t="inlineStr"/>
-      <c r="G35" s="8" t="inlineStr"/>
-      <c r="H35" s="8" t="inlineStr"/>
-    </row>
-    <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr"/>
+      <c r="D38" s="8" t="inlineStr"/>
+      <c r="E38" s="8" t="inlineStr"/>
+      <c r="F38" s="8" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr"/>
+      <c r="H38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39" ht="34" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>Checkout Step Completed</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>order_id</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
         <is>
           <t>ORD-20250401-9821</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr"/>
-      <c r="G36" s="9" t="inlineStr">
+      <c r="F39" s="9" t="inlineStr"/>
+      <c r="G39" s="9" t="inlineStr">
         <is>
           <t>Order ID.</t>
         </is>
       </c>
-      <c r="H36" s="9" t="inlineStr"/>
-    </row>
-    <row r="37" ht="34" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="H39" s="9" t="inlineStr"/>
+    </row>
+    <row r="40" ht="34" customHeight="1">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>Checkout Step Completed</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>step</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F40" s="9" t="inlineStr">
         <is>
           <t>1 | 2 | 3</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>Step number: 1=Address, 2=Delivery, 3=Payment.</t>
         </is>
       </c>
-      <c r="H37" s="9" t="inlineStr"/>
-    </row>
-    <row r="38" ht="34" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
+      <c r="H40" s="9" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>Checkout Step Completed</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>step_name</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
         <is>
           <t>address</t>
         </is>
       </c>
-      <c r="F38" s="9" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>address | delivery | payment</t>
         </is>
       </c>
-      <c r="G38" s="9" t="inlineStr">
+      <c r="G41" s="9" t="inlineStr">
         <is>
           <t>Step name slug.</t>
         </is>
       </c>
-      <c r="H38" s="9" t="inlineStr"/>
-    </row>
-    <row r="39" ht="34" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="H41" s="9" t="inlineStr"/>
+    </row>
+    <row r="42" ht="34" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Checkout Step Completed</t>
         </is>
       </c>
-      <c r="B39" s="10" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>payment_method</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>upi</t>
         </is>
       </c>
-      <c r="F39" s="10" t="inlineStr">
+      <c r="F42" s="10" t="inlineStr">
         <is>
           <t>upi | credit_card | debit_card | net_banking | cod | wallet</t>
         </is>
       </c>
-      <c r="G39" s="10" t="inlineStr">
+      <c r="G42" s="10" t="inlineStr">
         <is>
           <t>Populate on step 3 only.</t>
         </is>
       </c>
-      <c r="H39" s="10" t="inlineStr"/>
-    </row>
-    <row r="40" ht="34" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="H42" s="10" t="inlineStr"/>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Checkout Step Completed</t>
         </is>
       </c>
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>shipping_method</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
+      <c r="C43" s="10" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="D40" s="10" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E40" s="10" t="inlineStr">
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="F40" s="10" t="inlineStr">
+      <c r="F43" s="10" t="inlineStr">
         <is>
           <t>standard | express</t>
         </is>
       </c>
-      <c r="G40" s="10" t="inlineStr">
+      <c r="G43" s="10" t="inlineStr">
         <is>
           <t>Populate on step 2 only.</t>
         </is>
       </c>
-      <c r="H40" s="10" t="inlineStr"/>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>▶ Order Completed</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>Payment confirmed. Most critical revenue event. Segment Ecommerce standard.</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr"/>
-      <c r="D41" s="8" t="inlineStr"/>
-      <c r="E41" s="8" t="inlineStr"/>
-      <c r="F41" s="8" t="inlineStr"/>
-      <c r="G41" s="8" t="inlineStr"/>
-      <c r="H41" s="8" t="inlineStr"/>
-    </row>
-    <row r="42" ht="34" customHeight="1">
-      <c r="A42" s="9" t="inlineStr">
-        <is>
-          <t>Order Completed</t>
-        </is>
-      </c>
-      <c r="B42" s="9" t="inlineStr">
-        <is>
-          <t>order_id</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D42" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E42" s="9" t="inlineStr">
-        <is>
-          <t>ORD-20250401-9821</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="inlineStr"/>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>Final confirmed order ID. Must match backend.</t>
-        </is>
-      </c>
-      <c r="H42" s="9" t="inlineStr"/>
-    </row>
-    <row r="43" ht="34" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
-        <is>
-          <t>Order Completed</t>
-        </is>
-      </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>revenue</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>1518.20</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="inlineStr"/>
-      <c r="G43" s="9" t="inlineStr">
-        <is>
-          <t>Amount after discounts, before shipping. Used as Amplitude revenue property.</t>
-        </is>
-      </c>
-      <c r="H43" s="9" t="inlineStr"/>
+      <c r="H43" s="10" t="inlineStr"/>
     </row>
     <row r="44" ht="34" customHeight="1">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Order Completed</t>
+          <t>Checkout Step Completed</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>checkout_token</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
@@ -4404,55 +4488,39 @@
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>49.00</t>
-        </is>
-      </c>
-      <c r="F44" s="10" t="inlineStr"/>
+          <t>sh_9a8b7c6d</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="n"/>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>Shipping fee in INR.</t>
-        </is>
-      </c>
-      <c r="H44" s="10" t="inlineStr"/>
+          <t>Shopify checkout token. Same token as on Checkout Started.</t>
+        </is>
+      </c>
+      <c r="H44" s="10" t="n"/>
     </row>
     <row r="45" ht="34" customHeight="1">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t>Order Completed</t>
-        </is>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="inlineStr">
-        <is>
-          <t>1567.20</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="inlineStr"/>
-      <c r="G45" s="9" t="inlineStr">
-        <is>
-          <t>Grand total charged to customer including shipping.</t>
-        </is>
-      </c>
-      <c r="H45" s="9" t="inlineStr"/>
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>▶ Order Completed</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Payment confirmed. Most critical revenue event. Segment Ecommerce standard.</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr"/>
+      <c r="D45" s="8" t="inlineStr"/>
+      <c r="E45" s="8" t="inlineStr"/>
+      <c r="F45" s="8" t="inlineStr"/>
+      <c r="G45" s="8" t="inlineStr"/>
+      <c r="H45" s="8" t="inlineStr"/>
     </row>
     <row r="46" ht="34" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
@@ -4462,7 +4530,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>order_id</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
@@ -4477,54 +4545,50 @@
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>INR</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
+          <t>ORD-20250401-9821</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr"/>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>Always INR.</t>
+          <t>Final confirmed order ID. Must match backend.</t>
         </is>
       </c>
       <c r="H46" s="9" t="inlineStr"/>
     </row>
     <row r="47" ht="34" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>Order Completed</t>
         </is>
       </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>coupon</t>
-        </is>
-      </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E47" s="10" t="inlineStr">
-        <is>
-          <t>FIRST10</t>
-        </is>
-      </c>
-      <c r="F47" s="10" t="inlineStr"/>
-      <c r="G47" s="10" t="inlineStr">
-        <is>
-          <t>Coupon code used.</t>
-        </is>
-      </c>
-      <c r="H47" s="10" t="inlineStr"/>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>1518.20</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr"/>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>Amount after discounts, before shipping. Used as Amplitude revenue property.</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr"/>
     </row>
     <row r="48" ht="34" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
@@ -4534,7 +4598,7 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>discount</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
@@ -4549,13 +4613,13 @@
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>79.90</t>
+          <t>49.00</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr"/>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>Discount amount in INR.</t>
+          <t>Shipping fee in INR.</t>
         </is>
       </c>
       <c r="H48" s="10" t="inlineStr"/>
@@ -4568,7 +4632,7 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>payment_method</t>
+          <t>total</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -4578,22 +4642,18 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>upi</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>upi | credit_card | debit_card | net_banking | cod | wallet</t>
-        </is>
-      </c>
+          <t>1567.20</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr"/>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>Payment method confirmed.</t>
+          <t>Grand total charged to customer including shipping.</t>
         </is>
       </c>
       <c r="H49" s="9" t="inlineStr"/>
@@ -4606,7 +4666,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>num_items</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
@@ -4616,18 +4676,22 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="inlineStr"/>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>Total item count in order.</t>
+          <t>Always INR.</t>
         </is>
       </c>
       <c r="H50" s="9" t="inlineStr"/>
@@ -4640,37 +4704,273 @@
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
+          <t>coupon</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>FIRST10</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="inlineStr"/>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>Coupon code used.</t>
+        </is>
+      </c>
+      <c r="H51" s="10" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>Order Completed</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>discount</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>79.90</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr"/>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>Discount amount in INR.</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>Order Completed</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>payment_method</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>upi</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>upi | credit_card | debit_card | net_banking | cod | wallet</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>Payment method confirmed.</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>Order Completed</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>num_items</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr"/>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>Total item count in order.</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>Order Completed</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
           <t>is_first_order</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="D51" s="10" t="inlineStr">
+      <c r="D55" s="10" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="E51" s="10" t="inlineStr">
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F51" s="10" t="inlineStr">
+      <c r="F55" s="10" t="inlineStr">
         <is>
           <t>true | false</t>
         </is>
       </c>
-      <c r="G51" s="10" t="inlineStr">
+      <c r="G55" s="10" t="inlineStr">
         <is>
           <t>True if this is user's first ever order. Key new-user metric.</t>
         </is>
       </c>
-      <c r="H51" s="10" t="inlineStr">
+      <c r="H55" s="10" t="inlineStr">
         <is>
           <t>Derive: orders_count == 1 post-order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Order Completed</t>
+        </is>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>checkout_token</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>sh_9a8b7c6d</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Shopify checkout token.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Order Completed</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>[{...}]</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Segment spec products array.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Order Completed</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>273.96</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>18% GST on net revenue. Informational — not used in Amplitude revenue calc.</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6502,6 +6802,38 @@
       <c r="F13" s="10" t="inlineStr">
         <is>
           <t>Variant: control | treatment_a | treatment_b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>shop_name</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>kaliper-fashion.myshopify.com</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>context.shop_name</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Shopify store domain.</t>
         </is>
       </c>
     </row>

</xml_diff>